<commit_message>
Use active staff for workflow handoffs, add normal wear cause and include internal tickets in reporting
</commit_message>
<xml_diff>
--- a/public/templates/after-sales-import.xlsx
+++ b/public/templates/after-sales-import.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="售后记录单" sheetId="1" r:id="Re8438cf6274341e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例（不导入）" sheetId="2" r:id="R53314970bb8b492a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="3" r:id="Rbcd033ce55844f63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="售后记录单" sheetId="1" r:id="R56ea26f8abc6497b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例（不导入）" sheetId="2" r:id="Rc3bda2a2e80649d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="3" r:id="R33809bebcc80498f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -59,7 +59,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -136,6 +136,16 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border>
@@ -164,7 +174,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="54">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -303,6 +313,24 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -607,20 +635,20 @@
       <x:c r="B3" s="8" t="str">
         <x:v>项目名称 *</x:v>
       </x:c>
-      <x:c r="C3" s="42"/>
-      <x:c r="D3" s="42"/>
-      <x:c r="E3" s="42"/>
-      <x:c r="F3" s="42"/>
+      <x:c r="C3" s="48"/>
+      <x:c r="D3" s="48"/>
+      <x:c r="E3" s="48"/>
+      <x:c r="F3" s="48"/>
       <x:c r="G3" s="8" t="str">
         <x:v>客户名称 *</x:v>
       </x:c>
       <x:c r="H3" s="8" t="str">
         <x:v>客户名称 *</x:v>
       </x:c>
-      <x:c r="I3" s="42"/>
-      <x:c r="J3" s="42"/>
-      <x:c r="K3" s="42"/>
-      <x:c r="L3" s="42"/>
+      <x:c r="I3" s="48"/>
+      <x:c r="J3" s="48"/>
+      <x:c r="K3" s="48"/>
+      <x:c r="L3" s="48"/>
     </x:row>
     <x:row r="4" ht="31" customHeight="1">
       <x:c r="A4" s="8" t="str">
@@ -629,20 +657,20 @@
       <x:c r="B4" s="8" t="str">
         <x:v>原订单编号</x:v>
       </x:c>
-      <x:c r="C4" s="43"/>
-      <x:c r="D4" s="43"/>
-      <x:c r="E4" s="43"/>
-      <x:c r="F4" s="43"/>
+      <x:c r="C4" s="49"/>
+      <x:c r="D4" s="49"/>
+      <x:c r="E4" s="49"/>
+      <x:c r="F4" s="49"/>
       <x:c r="G4" s="8" t="str">
         <x:v>国家 / 地区</x:v>
       </x:c>
       <x:c r="H4" s="8" t="str">
         <x:v>国家 / 地区</x:v>
       </x:c>
-      <x:c r="I4" s="43"/>
-      <x:c r="J4" s="43"/>
-      <x:c r="K4" s="43"/>
-      <x:c r="L4" s="43"/>
+      <x:c r="I4" s="49"/>
+      <x:c r="J4" s="49"/>
+      <x:c r="K4" s="49"/>
+      <x:c r="L4" s="49"/>
     </x:row>
     <x:row r="5" ht="31" customHeight="1">
       <x:c r="A5" s="8" t="str">
@@ -651,24 +679,24 @@
       <x:c r="B5" s="8" t="str">
         <x:v>客户联系人</x:v>
       </x:c>
-      <x:c r="C5" s="43"/>
-      <x:c r="D5" s="43"/>
+      <x:c r="C5" s="49"/>
+      <x:c r="D5" s="49"/>
       <x:c r="E5" s="8" t="str">
         <x:v>联系电话</x:v>
       </x:c>
       <x:c r="F5" s="8" t="str">
         <x:v>联系电话</x:v>
       </x:c>
-      <x:c r="G5" s="43"/>
-      <x:c r="H5" s="43"/>
+      <x:c r="G5" s="49"/>
+      <x:c r="H5" s="49"/>
       <x:c r="I5" s="8" t="str">
         <x:v>WhatsApp / 微信</x:v>
       </x:c>
       <x:c r="J5" s="8" t="str">
         <x:v>WhatsApp / 微信</x:v>
       </x:c>
-      <x:c r="K5" s="43"/>
-      <x:c r="L5" s="43"/>
+      <x:c r="K5" s="49"/>
+      <x:c r="L5" s="49"/>
     </x:row>
     <x:row r="6" ht="31" customHeight="1">
       <x:c r="A6" s="8" t="str">
@@ -677,16 +705,16 @@
       <x:c r="B6" s="8" t="str">
         <x:v>项目详细地址</x:v>
       </x:c>
-      <x:c r="C6" s="43"/>
-      <x:c r="D6" s="43"/>
-      <x:c r="E6" s="43"/>
-      <x:c r="F6" s="43"/>
-      <x:c r="G6" s="43"/>
-      <x:c r="H6" s="43"/>
-      <x:c r="I6" s="43"/>
-      <x:c r="J6" s="43"/>
-      <x:c r="K6" s="43"/>
-      <x:c r="L6" s="43"/>
+      <x:c r="C6" s="49"/>
+      <x:c r="D6" s="49"/>
+      <x:c r="E6" s="49"/>
+      <x:c r="F6" s="49"/>
+      <x:c r="G6" s="49"/>
+      <x:c r="H6" s="49"/>
+      <x:c r="I6" s="49"/>
+      <x:c r="J6" s="49"/>
+      <x:c r="K6" s="49"/>
+      <x:c r="L6" s="49"/>
     </x:row>
     <x:row r="7" ht="31" customHeight="1">
       <x:c r="A7" s="8" t="str">
@@ -695,24 +723,24 @@
       <x:c r="B7" s="8" t="str">
         <x:v>报修日期</x:v>
       </x:c>
-      <x:c r="C7" s="44"/>
-      <x:c r="D7" s="44"/>
+      <x:c r="C7" s="50"/>
+      <x:c r="D7" s="50"/>
       <x:c r="E7" s="8" t="str">
         <x:v>保修资料填写方式</x:v>
       </x:c>
       <x:c r="F7" s="8" t="str">
         <x:v>保修资料填写方式</x:v>
       </x:c>
-      <x:c r="G7" s="43"/>
-      <x:c r="H7" s="43"/>
+      <x:c r="G7" s="49"/>
+      <x:c r="H7" s="49"/>
       <x:c r="I7" s="8" t="str">
         <x:v>保修截止日期</x:v>
       </x:c>
       <x:c r="J7" s="8" t="str">
         <x:v>保修截止日期</x:v>
       </x:c>
-      <x:c r="K7" s="44"/>
-      <x:c r="L7" s="44"/>
+      <x:c r="K7" s="50"/>
+      <x:c r="L7" s="50"/>
     </x:row>
     <x:row r="8" ht="31" customHeight="1">
       <x:c r="A8" s="8" t="str">
@@ -721,8 +749,8 @@
       <x:c r="B8" s="8" t="str">
         <x:v>保修开始日期</x:v>
       </x:c>
-      <x:c r="C8" s="44"/>
-      <x:c r="D8" s="44"/>
+      <x:c r="C8" s="50"/>
+      <x:c r="D8" s="50"/>
       <x:c r="E8" s="7" t="str">
         <x:v>保修状态 / 提醒</x:v>
       </x:c>
@@ -831,24 +859,24 @@
       <x:c r="B11" s="16" t="str">
         <x:v>产品名称 / 编号</x:v>
       </x:c>
-      <x:c r="C11" s="45"/>
-      <x:c r="D11" s="45"/>
+      <x:c r="C11" s="51"/>
+      <x:c r="D11" s="51"/>
       <x:c r="E11" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
-      <x:c r="G11" s="46"/>
-      <x:c r="H11" s="46"/>
+      <x:c r="G11" s="52"/>
+      <x:c r="H11" s="52"/>
       <x:c r="I11" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
       <x:c r="J11" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
-      <x:c r="K11" s="45"/>
-      <x:c r="L11" s="45"/>
+      <x:c r="K11" s="51"/>
+      <x:c r="L11" s="51"/>
     </x:row>
     <x:row r="12" ht="31" customHeight="1">
       <x:c r="A12" s="16" t="str">
@@ -857,24 +885,24 @@
       <x:c r="B12" s="16" t="str">
         <x:v>问题等级</x:v>
       </x:c>
-      <x:c r="C12" s="45"/>
-      <x:c r="D12" s="45"/>
+      <x:c r="C12" s="51"/>
+      <x:c r="D12" s="51"/>
       <x:c r="E12" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
-      <x:c r="G12" s="47"/>
-      <x:c r="H12" s="47"/>
+      <x:c r="G12" s="53"/>
+      <x:c r="H12" s="53"/>
       <x:c r="I12" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
       <x:c r="J12" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
-      <x:c r="K12" s="46"/>
-      <x:c r="L12" s="46"/>
+      <x:c r="K12" s="52"/>
+      <x:c r="L12" s="52"/>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="16" t="str">
@@ -883,16 +911,16 @@
       <x:c r="B13" s="16" t="str">
         <x:v>问题描述 *</x:v>
       </x:c>
-      <x:c r="C13" s="47"/>
-      <x:c r="D13" s="47"/>
-      <x:c r="E13" s="47"/>
-      <x:c r="F13" s="47"/>
-      <x:c r="G13" s="47"/>
-      <x:c r="H13" s="47"/>
-      <x:c r="I13" s="47"/>
-      <x:c r="J13" s="47"/>
-      <x:c r="K13" s="47"/>
-      <x:c r="L13" s="47"/>
+      <x:c r="C13" s="53"/>
+      <x:c r="D13" s="53"/>
+      <x:c r="E13" s="53"/>
+      <x:c r="F13" s="53"/>
+      <x:c r="G13" s="53"/>
+      <x:c r="H13" s="53"/>
+      <x:c r="I13" s="53"/>
+      <x:c r="J13" s="53"/>
+      <x:c r="K13" s="53"/>
+      <x:c r="L13" s="53"/>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="16" t="str">
@@ -901,18 +929,18 @@
       <x:c r="B14" s="16" t="str">
         <x:v>客户反馈 / 当前处理记录</x:v>
       </x:c>
-      <x:c r="C14" s="45"/>
-      <x:c r="D14" s="45"/>
-      <x:c r="E14" s="45"/>
-      <x:c r="F14" s="45"/>
-      <x:c r="G14" s="45"/>
-      <x:c r="H14" s="45"/>
+      <x:c r="C14" s="51"/>
+      <x:c r="D14" s="51"/>
+      <x:c r="E14" s="51"/>
+      <x:c r="F14" s="51"/>
+      <x:c r="G14" s="51"/>
+      <x:c r="H14" s="51"/>
       <x:c r="I14" s="22" t="str">
         <x:v>售后原因</x:v>
       </x:c>
       <x:c r="J14" s="22"/>
-      <x:c r="K14" s="45"/>
-      <x:c r="L14" s="45"/>
+      <x:c r="K14" s="51"/>
+      <x:c r="L14" s="51"/>
     </x:row>
     <x:row r="15" ht="135" customHeight="1">
       <x:c r="A15" s="16" t="str">
@@ -921,20 +949,20 @@
       <x:c r="B15" s="16" t="str">
         <x:v>附件提供方式</x:v>
       </x:c>
-      <x:c r="C15" s="45"/>
-      <x:c r="D15" s="45"/>
+      <x:c r="C15" s="51"/>
+      <x:c r="D15" s="51"/>
       <x:c r="E15" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
       <x:c r="F15" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
-      <x:c r="G15" s="45"/>
-      <x:c r="H15" s="45"/>
-      <x:c r="I15" s="45"/>
-      <x:c r="J15" s="45"/>
-      <x:c r="K15" s="45"/>
-      <x:c r="L15" s="45"/>
+      <x:c r="G15" s="51"/>
+      <x:c r="H15" s="51"/>
+      <x:c r="I15" s="51"/>
+      <x:c r="J15" s="51"/>
+      <x:c r="K15" s="51"/>
+      <x:c r="L15" s="51"/>
     </x:row>
     <x:row r="16" ht="31" customHeight="1">
       <x:c r="A16" s="16" t="str">
@@ -943,24 +971,24 @@
       <x:c r="B16" s="16" t="str">
         <x:v>当前阶段</x:v>
       </x:c>
-      <x:c r="C16" s="45"/>
-      <x:c r="D16" s="45"/>
+      <x:c r="C16" s="51"/>
+      <x:c r="D16" s="51"/>
       <x:c r="E16" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
       <x:c r="F16" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
-      <x:c r="G16" s="46"/>
-      <x:c r="H16" s="46"/>
+      <x:c r="G16" s="52"/>
+      <x:c r="H16" s="52"/>
       <x:c r="I16" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
       <x:c r="J16" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
-      <x:c r="K16" s="45"/>
-      <x:c r="L16" s="45"/>
+      <x:c r="K16" s="51"/>
+      <x:c r="L16" s="51"/>
     </x:row>
     <x:row r="17" ht="31" customHeight="1">
       <x:c r="A17" s="16" t="str">
@@ -969,24 +997,24 @@
       <x:c r="B17" s="16" t="str">
         <x:v>商务</x:v>
       </x:c>
-      <x:c r="C17" s="45"/>
-      <x:c r="D17" s="45"/>
+      <x:c r="C17" s="51"/>
+      <x:c r="D17" s="51"/>
       <x:c r="E17" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
       <x:c r="F17" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
-      <x:c r="G17" s="45"/>
-      <x:c r="H17" s="45"/>
+      <x:c r="G17" s="51"/>
+      <x:c r="H17" s="51"/>
       <x:c r="I17" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
       <x:c r="J17" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
-      <x:c r="K17" s="45"/>
-      <x:c r="L17" s="45"/>
+      <x:c r="K17" s="51"/>
+      <x:c r="L17" s="51"/>
     </x:row>
     <x:row r="18" ht="31" customHeight="1">
       <x:c r="A18" s="16" t="str">
@@ -995,24 +1023,24 @@
       <x:c r="B18" s="16" t="str">
         <x:v>安装人员</x:v>
       </x:c>
-      <x:c r="C18" s="45"/>
-      <x:c r="D18" s="45"/>
+      <x:c r="C18" s="51"/>
+      <x:c r="D18" s="51"/>
       <x:c r="E18" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
       <x:c r="F18" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
-      <x:c r="G18" s="45"/>
-      <x:c r="H18" s="45"/>
+      <x:c r="G18" s="51"/>
+      <x:c r="H18" s="51"/>
       <x:c r="I18" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
       <x:c r="J18" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
-      <x:c r="K18" s="45"/>
-      <x:c r="L18" s="45"/>
+      <x:c r="K18" s="51"/>
+      <x:c r="L18" s="51"/>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="15" t="str">
@@ -1059,24 +1087,24 @@
       <x:c r="B20" s="16" t="str">
         <x:v>产品名称 / 编号</x:v>
       </x:c>
-      <x:c r="C20" s="45"/>
-      <x:c r="D20" s="45"/>
+      <x:c r="C20" s="51"/>
+      <x:c r="D20" s="51"/>
       <x:c r="E20" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
       <x:c r="F20" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
-      <x:c r="G20" s="46"/>
-      <x:c r="H20" s="46"/>
+      <x:c r="G20" s="52"/>
+      <x:c r="H20" s="52"/>
       <x:c r="I20" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
       <x:c r="J20" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
-      <x:c r="K20" s="45"/>
-      <x:c r="L20" s="45"/>
+      <x:c r="K20" s="51"/>
+      <x:c r="L20" s="51"/>
     </x:row>
     <x:row r="21" ht="31" customHeight="1">
       <x:c r="A21" s="16" t="str">
@@ -1085,24 +1113,24 @@
       <x:c r="B21" s="16" t="str">
         <x:v>问题等级</x:v>
       </x:c>
-      <x:c r="C21" s="45"/>
-      <x:c r="D21" s="45"/>
+      <x:c r="C21" s="51"/>
+      <x:c r="D21" s="51"/>
       <x:c r="E21" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
       <x:c r="F21" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
-      <x:c r="G21" s="47"/>
-      <x:c r="H21" s="47"/>
+      <x:c r="G21" s="53"/>
+      <x:c r="H21" s="53"/>
       <x:c r="I21" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
       <x:c r="J21" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
-      <x:c r="K21" s="46"/>
-      <x:c r="L21" s="46"/>
+      <x:c r="K21" s="52"/>
+      <x:c r="L21" s="52"/>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="16" t="str">
@@ -1111,16 +1139,16 @@
       <x:c r="B22" s="16" t="str">
         <x:v>问题描述 *</x:v>
       </x:c>
-      <x:c r="C22" s="47"/>
-      <x:c r="D22" s="47"/>
-      <x:c r="E22" s="47"/>
-      <x:c r="F22" s="47"/>
-      <x:c r="G22" s="47"/>
-      <x:c r="H22" s="47"/>
-      <x:c r="I22" s="47"/>
-      <x:c r="J22" s="47"/>
-      <x:c r="K22" s="47"/>
-      <x:c r="L22" s="47"/>
+      <x:c r="C22" s="53"/>
+      <x:c r="D22" s="53"/>
+      <x:c r="E22" s="53"/>
+      <x:c r="F22" s="53"/>
+      <x:c r="G22" s="53"/>
+      <x:c r="H22" s="53"/>
+      <x:c r="I22" s="53"/>
+      <x:c r="J22" s="53"/>
+      <x:c r="K22" s="53"/>
+      <x:c r="L22" s="53"/>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" s="16" t="str">
@@ -1129,18 +1157,18 @@
       <x:c r="B23" s="16" t="str">
         <x:v>客户反馈 / 当前处理记录</x:v>
       </x:c>
-      <x:c r="C23" s="45"/>
-      <x:c r="D23" s="45"/>
-      <x:c r="E23" s="45"/>
-      <x:c r="F23" s="45"/>
-      <x:c r="G23" s="45"/>
-      <x:c r="H23" s="45"/>
+      <x:c r="C23" s="51"/>
+      <x:c r="D23" s="51"/>
+      <x:c r="E23" s="51"/>
+      <x:c r="F23" s="51"/>
+      <x:c r="G23" s="51"/>
+      <x:c r="H23" s="51"/>
       <x:c r="I23" s="22" t="str">
         <x:v>售后原因</x:v>
       </x:c>
       <x:c r="J23" s="22"/>
-      <x:c r="K23" s="45"/>
-      <x:c r="L23" s="45"/>
+      <x:c r="K23" s="51"/>
+      <x:c r="L23" s="51"/>
     </x:row>
     <x:row r="24" ht="135" customHeight="1">
       <x:c r="A24" s="16" t="str">
@@ -1149,20 +1177,20 @@
       <x:c r="B24" s="16" t="str">
         <x:v>附件提供方式</x:v>
       </x:c>
-      <x:c r="C24" s="45"/>
-      <x:c r="D24" s="45"/>
+      <x:c r="C24" s="51"/>
+      <x:c r="D24" s="51"/>
       <x:c r="E24" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
       <x:c r="F24" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
-      <x:c r="G24" s="45"/>
-      <x:c r="H24" s="45"/>
-      <x:c r="I24" s="45"/>
-      <x:c r="J24" s="45"/>
-      <x:c r="K24" s="45"/>
-      <x:c r="L24" s="45"/>
+      <x:c r="G24" s="51"/>
+      <x:c r="H24" s="51"/>
+      <x:c r="I24" s="51"/>
+      <x:c r="J24" s="51"/>
+      <x:c r="K24" s="51"/>
+      <x:c r="L24" s="51"/>
     </x:row>
     <x:row r="25" ht="31" customHeight="1">
       <x:c r="A25" s="16" t="str">
@@ -1171,24 +1199,24 @@
       <x:c r="B25" s="16" t="str">
         <x:v>当前阶段</x:v>
       </x:c>
-      <x:c r="C25" s="45"/>
-      <x:c r="D25" s="45"/>
+      <x:c r="C25" s="51"/>
+      <x:c r="D25" s="51"/>
       <x:c r="E25" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
       <x:c r="F25" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
-      <x:c r="G25" s="46"/>
-      <x:c r="H25" s="46"/>
+      <x:c r="G25" s="52"/>
+      <x:c r="H25" s="52"/>
       <x:c r="I25" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
       <x:c r="J25" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
-      <x:c r="K25" s="45"/>
-      <x:c r="L25" s="45"/>
+      <x:c r="K25" s="51"/>
+      <x:c r="L25" s="51"/>
     </x:row>
     <x:row r="26" ht="31" customHeight="1">
       <x:c r="A26" s="16" t="str">
@@ -1197,24 +1225,24 @@
       <x:c r="B26" s="16" t="str">
         <x:v>商务</x:v>
       </x:c>
-      <x:c r="C26" s="45"/>
-      <x:c r="D26" s="45"/>
+      <x:c r="C26" s="51"/>
+      <x:c r="D26" s="51"/>
       <x:c r="E26" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
       <x:c r="F26" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
-      <x:c r="G26" s="45"/>
-      <x:c r="H26" s="45"/>
+      <x:c r="G26" s="51"/>
+      <x:c r="H26" s="51"/>
       <x:c r="I26" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
       <x:c r="J26" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
-      <x:c r="K26" s="45"/>
-      <x:c r="L26" s="45"/>
+      <x:c r="K26" s="51"/>
+      <x:c r="L26" s="51"/>
     </x:row>
     <x:row r="27" ht="31" customHeight="1">
       <x:c r="A27" s="16" t="str">
@@ -1223,24 +1251,24 @@
       <x:c r="B27" s="16" t="str">
         <x:v>安装人员</x:v>
       </x:c>
-      <x:c r="C27" s="45"/>
-      <x:c r="D27" s="45"/>
+      <x:c r="C27" s="51"/>
+      <x:c r="D27" s="51"/>
       <x:c r="E27" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
       <x:c r="F27" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
-      <x:c r="G27" s="45"/>
-      <x:c r="H27" s="45"/>
+      <x:c r="G27" s="51"/>
+      <x:c r="H27" s="51"/>
       <x:c r="I27" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
       <x:c r="J27" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
-      <x:c r="K27" s="45"/>
-      <x:c r="L27" s="45"/>
+      <x:c r="K27" s="51"/>
+      <x:c r="L27" s="51"/>
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="15" t="str">
@@ -1287,24 +1315,24 @@
       <x:c r="B29" s="16" t="str">
         <x:v>产品名称 / 编号</x:v>
       </x:c>
-      <x:c r="C29" s="45"/>
-      <x:c r="D29" s="45"/>
+      <x:c r="C29" s="51"/>
+      <x:c r="D29" s="51"/>
       <x:c r="E29" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
       <x:c r="F29" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
-      <x:c r="G29" s="46"/>
-      <x:c r="H29" s="46"/>
+      <x:c r="G29" s="52"/>
+      <x:c r="H29" s="52"/>
       <x:c r="I29" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
       <x:c r="J29" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
-      <x:c r="K29" s="45"/>
-      <x:c r="L29" s="45"/>
+      <x:c r="K29" s="51"/>
+      <x:c r="L29" s="51"/>
     </x:row>
     <x:row r="30" ht="31" customHeight="1">
       <x:c r="A30" s="16" t="str">
@@ -1313,24 +1341,24 @@
       <x:c r="B30" s="16" t="str">
         <x:v>问题等级</x:v>
       </x:c>
-      <x:c r="C30" s="45"/>
-      <x:c r="D30" s="45"/>
+      <x:c r="C30" s="51"/>
+      <x:c r="D30" s="51"/>
       <x:c r="E30" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
       <x:c r="F30" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
-      <x:c r="G30" s="47"/>
-      <x:c r="H30" s="47"/>
+      <x:c r="G30" s="53"/>
+      <x:c r="H30" s="53"/>
       <x:c r="I30" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
       <x:c r="J30" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
-      <x:c r="K30" s="46"/>
-      <x:c r="L30" s="46"/>
+      <x:c r="K30" s="52"/>
+      <x:c r="L30" s="52"/>
     </x:row>
     <x:row r="31" ht="48" customHeight="1">
       <x:c r="A31" s="16" t="str">
@@ -1339,16 +1367,16 @@
       <x:c r="B31" s="16" t="str">
         <x:v>问题描述 *</x:v>
       </x:c>
-      <x:c r="C31" s="47"/>
-      <x:c r="D31" s="47"/>
-      <x:c r="E31" s="47"/>
-      <x:c r="F31" s="47"/>
-      <x:c r="G31" s="47"/>
-      <x:c r="H31" s="47"/>
-      <x:c r="I31" s="47"/>
-      <x:c r="J31" s="47"/>
-      <x:c r="K31" s="47"/>
-      <x:c r="L31" s="47"/>
+      <x:c r="C31" s="53"/>
+      <x:c r="D31" s="53"/>
+      <x:c r="E31" s="53"/>
+      <x:c r="F31" s="53"/>
+      <x:c r="G31" s="53"/>
+      <x:c r="H31" s="53"/>
+      <x:c r="I31" s="53"/>
+      <x:c r="J31" s="53"/>
+      <x:c r="K31" s="53"/>
+      <x:c r="L31" s="53"/>
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
       <x:c r="A32" s="16" t="str">
@@ -1357,18 +1385,18 @@
       <x:c r="B32" s="16" t="str">
         <x:v>客户反馈 / 当前处理记录</x:v>
       </x:c>
-      <x:c r="C32" s="45"/>
-      <x:c r="D32" s="45"/>
-      <x:c r="E32" s="45"/>
-      <x:c r="F32" s="45"/>
-      <x:c r="G32" s="45"/>
-      <x:c r="H32" s="45"/>
+      <x:c r="C32" s="51"/>
+      <x:c r="D32" s="51"/>
+      <x:c r="E32" s="51"/>
+      <x:c r="F32" s="51"/>
+      <x:c r="G32" s="51"/>
+      <x:c r="H32" s="51"/>
       <x:c r="I32" s="22" t="str">
         <x:v>售后原因</x:v>
       </x:c>
       <x:c r="J32" s="22"/>
-      <x:c r="K32" s="45"/>
-      <x:c r="L32" s="45"/>
+      <x:c r="K32" s="51"/>
+      <x:c r="L32" s="51"/>
     </x:row>
     <x:row r="33" ht="135" customHeight="1">
       <x:c r="A33" s="16" t="str">
@@ -1377,20 +1405,20 @@
       <x:c r="B33" s="16" t="str">
         <x:v>附件提供方式</x:v>
       </x:c>
-      <x:c r="C33" s="45"/>
-      <x:c r="D33" s="45"/>
+      <x:c r="C33" s="51"/>
+      <x:c r="D33" s="51"/>
       <x:c r="E33" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
       <x:c r="F33" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
-      <x:c r="G33" s="45"/>
-      <x:c r="H33" s="45"/>
-      <x:c r="I33" s="45"/>
-      <x:c r="J33" s="45"/>
-      <x:c r="K33" s="45"/>
-      <x:c r="L33" s="45"/>
+      <x:c r="G33" s="51"/>
+      <x:c r="H33" s="51"/>
+      <x:c r="I33" s="51"/>
+      <x:c r="J33" s="51"/>
+      <x:c r="K33" s="51"/>
+      <x:c r="L33" s="51"/>
     </x:row>
     <x:row r="34" ht="31" customHeight="1">
       <x:c r="A34" s="16" t="str">
@@ -1399,24 +1427,24 @@
       <x:c r="B34" s="16" t="str">
         <x:v>当前阶段</x:v>
       </x:c>
-      <x:c r="C34" s="45"/>
-      <x:c r="D34" s="45"/>
+      <x:c r="C34" s="51"/>
+      <x:c r="D34" s="51"/>
       <x:c r="E34" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
       <x:c r="F34" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
-      <x:c r="G34" s="46"/>
-      <x:c r="H34" s="46"/>
+      <x:c r="G34" s="52"/>
+      <x:c r="H34" s="52"/>
       <x:c r="I34" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
       <x:c r="J34" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
-      <x:c r="K34" s="45"/>
-      <x:c r="L34" s="45"/>
+      <x:c r="K34" s="51"/>
+      <x:c r="L34" s="51"/>
     </x:row>
     <x:row r="35" ht="31" customHeight="1">
       <x:c r="A35" s="16" t="str">
@@ -1425,24 +1453,24 @@
       <x:c r="B35" s="16" t="str">
         <x:v>商务</x:v>
       </x:c>
-      <x:c r="C35" s="45"/>
-      <x:c r="D35" s="45"/>
+      <x:c r="C35" s="51"/>
+      <x:c r="D35" s="51"/>
       <x:c r="E35" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
       <x:c r="F35" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
-      <x:c r="G35" s="45"/>
-      <x:c r="H35" s="45"/>
+      <x:c r="G35" s="51"/>
+      <x:c r="H35" s="51"/>
       <x:c r="I35" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
       <x:c r="J35" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
-      <x:c r="K35" s="45"/>
-      <x:c r="L35" s="45"/>
+      <x:c r="K35" s="51"/>
+      <x:c r="L35" s="51"/>
     </x:row>
     <x:row r="36" ht="31" customHeight="1">
       <x:c r="A36" s="16" t="str">
@@ -1451,24 +1479,24 @@
       <x:c r="B36" s="16" t="str">
         <x:v>安装人员</x:v>
       </x:c>
-      <x:c r="C36" s="45"/>
-      <x:c r="D36" s="45"/>
+      <x:c r="C36" s="51"/>
+      <x:c r="D36" s="51"/>
       <x:c r="E36" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
       <x:c r="F36" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
-      <x:c r="G36" s="45"/>
-      <x:c r="H36" s="45"/>
+      <x:c r="G36" s="51"/>
+      <x:c r="H36" s="51"/>
       <x:c r="I36" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
       <x:c r="J36" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
-      <x:c r="K36" s="45"/>
-      <x:c r="L36" s="45"/>
+      <x:c r="K36" s="51"/>
+      <x:c r="L36" s="51"/>
     </x:row>
     <x:row r="37" ht="27" customHeight="1">
       <x:c r="A37" s="6" t="str">
@@ -1714,7 +1742,7 @@
       <x:formula1>"待评估,S,A,B,C"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K14:L14">
-      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏"</x:formula1>
+      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏,正常损耗"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C15:D15">
       <x:formula1>"上传照片 / 视频,照片 / 视频链接"</x:formula1>
@@ -1735,7 +1763,7 @@
       <x:formula1>"待评估,S,A,B,C"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K23:L23">
-      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏"</x:formula1>
+      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏,正常损耗"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C24:D24">
       <x:formula1>"上传照片 / 视频,照片 / 视频链接"</x:formula1>
@@ -1756,7 +1784,7 @@
       <x:formula1>"待评估,S,A,B,C"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K32:L32">
-      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏"</x:formula1>
+      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏,正常损耗"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C33:D33">
       <x:formula1>"上传照片 / 视频,照片 / 视频链接"</x:formula1>
@@ -1879,24 +1907,24 @@
       <x:c r="B3" s="8" t="str">
         <x:v>项目名称 *</x:v>
       </x:c>
-      <x:c r="C3" s="42" t="str">
+      <x:c r="C3" s="48" t="str">
         <x:v>示例项目 A</x:v>
       </x:c>
-      <x:c r="D3" s="42"/>
-      <x:c r="E3" s="42"/>
-      <x:c r="F3" s="42"/>
+      <x:c r="D3" s="48"/>
+      <x:c r="E3" s="48"/>
+      <x:c r="F3" s="48"/>
       <x:c r="G3" s="8" t="str">
         <x:v>客户名称 *</x:v>
       </x:c>
       <x:c r="H3" s="8" t="str">
         <x:v>客户名称 *</x:v>
       </x:c>
-      <x:c r="I3" s="42" t="str">
+      <x:c r="I3" s="48" t="str">
         <x:v>示例连锁客户 A</x:v>
       </x:c>
-      <x:c r="J3" s="42"/>
-      <x:c r="K3" s="42"/>
-      <x:c r="L3" s="42"/>
+      <x:c r="J3" s="48"/>
+      <x:c r="K3" s="48"/>
+      <x:c r="L3" s="48"/>
     </x:row>
     <x:row r="4" ht="31" customHeight="1">
       <x:c r="A4" s="8" t="str">
@@ -1905,24 +1933,24 @@
       <x:c r="B4" s="8" t="str">
         <x:v>原订单编号</x:v>
       </x:c>
-      <x:c r="C4" s="43" t="str">
+      <x:c r="C4" s="49" t="str">
         <x:v>YW-ORD-001</x:v>
       </x:c>
-      <x:c r="D4" s="43"/>
-      <x:c r="E4" s="43"/>
-      <x:c r="F4" s="43"/>
+      <x:c r="D4" s="49"/>
+      <x:c r="E4" s="49"/>
+      <x:c r="F4" s="49"/>
       <x:c r="G4" s="8" t="str">
         <x:v>国家 / 地区</x:v>
       </x:c>
       <x:c r="H4" s="8" t="str">
         <x:v>国家 / 地区</x:v>
       </x:c>
-      <x:c r="I4" s="43" t="str">
+      <x:c r="I4" s="49" t="str">
         <x:v>阿联酋</x:v>
       </x:c>
-      <x:c r="J4" s="43"/>
-      <x:c r="K4" s="43"/>
-      <x:c r="L4" s="43"/>
+      <x:c r="J4" s="49"/>
+      <x:c r="K4" s="49"/>
+      <x:c r="L4" s="49"/>
     </x:row>
     <x:row r="5" ht="31" customHeight="1">
       <x:c r="A5" s="8" t="str">
@@ -1931,28 +1959,28 @@
       <x:c r="B5" s="8" t="str">
         <x:v>客户联系人</x:v>
       </x:c>
-      <x:c r="C5" s="43" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>示例联系人 A</x:v>
       </x:c>
-      <x:c r="D5" s="43"/>
+      <x:c r="D5" s="49"/>
       <x:c r="E5" s="8" t="str">
         <x:v>联系电话</x:v>
       </x:c>
       <x:c r="F5" s="8" t="str">
         <x:v>联系电话</x:v>
       </x:c>
-      <x:c r="G5" s="43" t="str"/>
-      <x:c r="H5" s="43"/>
+      <x:c r="G5" s="49" t="str"/>
+      <x:c r="H5" s="49"/>
       <x:c r="I5" s="8" t="str">
         <x:v>WhatsApp / 微信</x:v>
       </x:c>
       <x:c r="J5" s="8" t="str">
         <x:v>WhatsApp / 微信</x:v>
       </x:c>
-      <x:c r="K5" s="43" t="str">
+      <x:c r="K5" s="49" t="str">
         <x:v>示例微信号（请替换）</x:v>
       </x:c>
-      <x:c r="L5" s="43"/>
+      <x:c r="L5" s="49"/>
     </x:row>
     <x:row r="6" ht="31" customHeight="1">
       <x:c r="A6" s="8" t="str">
@@ -1961,18 +1989,18 @@
       <x:c r="B6" s="8" t="str">
         <x:v>项目详细地址</x:v>
       </x:c>
-      <x:c r="C6" s="43" t="str">
+      <x:c r="C6" s="49" t="str">
         <x:v>示例项目现场地址（请替换为实际地址）</x:v>
       </x:c>
-      <x:c r="D6" s="43"/>
-      <x:c r="E6" s="43"/>
-      <x:c r="F6" s="43"/>
-      <x:c r="G6" s="43"/>
-      <x:c r="H6" s="43"/>
-      <x:c r="I6" s="43"/>
-      <x:c r="J6" s="43"/>
-      <x:c r="K6" s="43"/>
-      <x:c r="L6" s="43"/>
+      <x:c r="D6" s="49"/>
+      <x:c r="E6" s="49"/>
+      <x:c r="F6" s="49"/>
+      <x:c r="G6" s="49"/>
+      <x:c r="H6" s="49"/>
+      <x:c r="I6" s="49"/>
+      <x:c r="J6" s="49"/>
+      <x:c r="K6" s="49"/>
+      <x:c r="L6" s="49"/>
     </x:row>
     <x:row r="7" ht="31" customHeight="1">
       <x:c r="A7" s="8" t="str">
@@ -1981,30 +2009,30 @@
       <x:c r="B7" s="8" t="str">
         <x:v>报修日期</x:v>
       </x:c>
-      <x:c r="C7" s="44" t="d">
+      <x:c r="C7" s="50" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="D7" s="44"/>
+      <x:c r="D7" s="50"/>
       <x:c r="E7" s="8" t="str">
         <x:v>保修资料填写方式</x:v>
       </x:c>
       <x:c r="F7" s="8" t="str">
         <x:v>保修资料填写方式</x:v>
       </x:c>
-      <x:c r="G7" s="43" t="str">
+      <x:c r="G7" s="49" t="str">
         <x:v>手工填写</x:v>
       </x:c>
-      <x:c r="H7" s="43"/>
+      <x:c r="H7" s="49"/>
       <x:c r="I7" s="8" t="str">
         <x:v>保修截止日期</x:v>
       </x:c>
       <x:c r="J7" s="8" t="str">
         <x:v>保修截止日期</x:v>
       </x:c>
-      <x:c r="K7" s="44" t="d">
+      <x:c r="K7" s="50" t="d">
         <x:v>2026-12-31T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="L7" s="44"/>
+      <x:c r="L7" s="50"/>
     </x:row>
     <x:row r="8" ht="31" customHeight="1">
       <x:c r="A8" s="8" t="str">
@@ -2013,10 +2041,10 @@
       <x:c r="B8" s="8" t="str">
         <x:v>保修开始日期</x:v>
       </x:c>
-      <x:c r="C8" s="44" t="d">
+      <x:c r="C8" s="50" t="d">
         <x:v>2026-01-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="D8" s="44"/>
+      <x:c r="D8" s="50"/>
       <x:c r="E8" s="7" t="str">
         <x:v>保修状态 / 提醒</x:v>
       </x:c>
@@ -2125,30 +2153,30 @@
       <x:c r="B11" s="16" t="str">
         <x:v>产品名称 / 编号</x:v>
       </x:c>
-      <x:c r="C11" s="45" t="str">
+      <x:c r="C11" s="51" t="str">
         <x:v>电机 M01</x:v>
       </x:c>
-      <x:c r="D11" s="45"/>
+      <x:c r="D11" s="51"/>
       <x:c r="E11" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
-      <x:c r="G11" s="46" t="d">
+      <x:c r="G11" s="52" t="d">
         <x:v>2026-01-10T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="H11" s="46"/>
+      <x:c r="H11" s="52"/>
       <x:c r="I11" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
       <x:c r="J11" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
-      <x:c r="K11" s="45" t="str">
+      <x:c r="K11" s="51" t="str">
         <x:v>设备故障</x:v>
       </x:c>
-      <x:c r="L11" s="45"/>
+      <x:c r="L11" s="51"/>
     </x:row>
     <x:row r="12" ht="31" customHeight="1">
       <x:c r="A12" s="16" t="str">
@@ -2157,30 +2185,30 @@
       <x:c r="B12" s="16" t="str">
         <x:v>问题等级</x:v>
       </x:c>
-      <x:c r="C12" s="45" t="str">
+      <x:c r="C12" s="51" t="str">
         <x:v>待评估</x:v>
       </x:c>
-      <x:c r="D12" s="45"/>
+      <x:c r="D12" s="51"/>
       <x:c r="E12" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
-      <x:c r="G12" s="47" t="str">
+      <x:c r="G12" s="53" t="str">
         <x:v>张售后</x:v>
       </x:c>
-      <x:c r="H12" s="47"/>
+      <x:c r="H12" s="53"/>
       <x:c r="I12" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
       <x:c r="J12" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
-      <x:c r="K12" s="46" t="d">
+      <x:c r="K12" s="52" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="L12" s="46"/>
+      <x:c r="L12" s="52"/>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="16" t="str">
@@ -2189,18 +2217,18 @@
       <x:c r="B13" s="16" t="str">
         <x:v>问题描述 *</x:v>
       </x:c>
-      <x:c r="C13" s="47" t="str">
+      <x:c r="C13" s="53" t="str">
         <x:v>开机后电机有异响，连续出现两次，已暂停使用。</x:v>
       </x:c>
-      <x:c r="D13" s="47"/>
-      <x:c r="E13" s="47"/>
-      <x:c r="F13" s="47"/>
-      <x:c r="G13" s="47"/>
-      <x:c r="H13" s="47"/>
-      <x:c r="I13" s="47"/>
-      <x:c r="J13" s="47"/>
-      <x:c r="K13" s="47"/>
-      <x:c r="L13" s="47"/>
+      <x:c r="D13" s="53"/>
+      <x:c r="E13" s="53"/>
+      <x:c r="F13" s="53"/>
+      <x:c r="G13" s="53"/>
+      <x:c r="H13" s="53"/>
+      <x:c r="I13" s="53"/>
+      <x:c r="J13" s="53"/>
+      <x:c r="K13" s="53"/>
+      <x:c r="L13" s="53"/>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="16" t="str">
@@ -2209,20 +2237,20 @@
       <x:c r="B14" s="16" t="str">
         <x:v>客户反馈 / 当前处理记录</x:v>
       </x:c>
-      <x:c r="C14" s="45" t="str">
+      <x:c r="C14" s="51" t="str">
         <x:v>已联系客户收集视频，等待技术评估。</x:v>
       </x:c>
-      <x:c r="D14" s="45"/>
-      <x:c r="E14" s="45"/>
-      <x:c r="F14" s="45"/>
-      <x:c r="G14" s="45"/>
-      <x:c r="H14" s="45"/>
+      <x:c r="D14" s="51"/>
+      <x:c r="E14" s="51"/>
+      <x:c r="F14" s="51"/>
+      <x:c r="G14" s="51"/>
+      <x:c r="H14" s="51"/>
       <x:c r="I14" s="22" t="str">
         <x:v>售后原因</x:v>
       </x:c>
       <x:c r="J14" s="22"/>
-      <x:c r="K14" s="45"/>
-      <x:c r="L14" s="45"/>
+      <x:c r="K14" s="51"/>
+      <x:c r="L14" s="51"/>
     </x:row>
     <x:row r="15" ht="135" customHeight="1">
       <x:c r="A15" s="16" t="str">
@@ -2231,22 +2259,22 @@
       <x:c r="B15" s="16" t="str">
         <x:v>附件提供方式</x:v>
       </x:c>
-      <x:c r="C15" s="45" t="str">
+      <x:c r="C15" s="51" t="str">
         <x:v>上传照片 / 视频</x:v>
       </x:c>
-      <x:c r="D15" s="45"/>
+      <x:c r="D15" s="51"/>
       <x:c r="E15" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
       <x:c r="F15" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
-      <x:c r="G15" s="45" t="str"/>
-      <x:c r="H15" s="45"/>
-      <x:c r="I15" s="45"/>
-      <x:c r="J15" s="45"/>
-      <x:c r="K15" s="45"/>
-      <x:c r="L15" s="45"/>
+      <x:c r="G15" s="51" t="str"/>
+      <x:c r="H15" s="51"/>
+      <x:c r="I15" s="51"/>
+      <x:c r="J15" s="51"/>
+      <x:c r="K15" s="51"/>
+      <x:c r="L15" s="51"/>
     </x:row>
     <x:row r="16" ht="31" customHeight="1">
       <x:c r="A16" s="16" t="str">
@@ -2255,28 +2283,28 @@
       <x:c r="B16" s="16" t="str">
         <x:v>当前阶段</x:v>
       </x:c>
-      <x:c r="C16" s="45" t="str">
+      <x:c r="C16" s="51" t="str">
         <x:v>审核</x:v>
       </x:c>
-      <x:c r="D16" s="45"/>
+      <x:c r="D16" s="51"/>
       <x:c r="E16" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
       <x:c r="F16" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
-      <x:c r="G16" s="46"/>
-      <x:c r="H16" s="46"/>
+      <x:c r="G16" s="52"/>
+      <x:c r="H16" s="52"/>
       <x:c r="I16" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
       <x:c r="J16" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
-      <x:c r="K16" s="45" t="str">
+      <x:c r="K16" s="51" t="str">
         <x:v>确认电机异响原因</x:v>
       </x:c>
-      <x:c r="L16" s="45"/>
+      <x:c r="L16" s="51"/>
     </x:row>
     <x:row r="17" ht="31" customHeight="1">
       <x:c r="A17" s="16" t="str">
@@ -2285,30 +2313,30 @@
       <x:c r="B17" s="16" t="str">
         <x:v>商务</x:v>
       </x:c>
-      <x:c r="C17" s="45" t="str">
+      <x:c r="C17" s="51" t="str">
         <x:v>林商务</x:v>
       </x:c>
-      <x:c r="D17" s="45"/>
+      <x:c r="D17" s="51"/>
       <x:c r="E17" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
       <x:c r="F17" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
-      <x:c r="G17" s="45" t="str">
+      <x:c r="G17" s="51" t="str">
         <x:v>陈设计</x:v>
       </x:c>
-      <x:c r="H17" s="45"/>
+      <x:c r="H17" s="51"/>
       <x:c r="I17" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
       <x:c r="J17" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
-      <x:c r="K17" s="45" t="str">
+      <x:c r="K17" s="51" t="str">
         <x:v>周工程</x:v>
       </x:c>
-      <x:c r="L17" s="45"/>
+      <x:c r="L17" s="51"/>
     </x:row>
     <x:row r="18" ht="31" customHeight="1">
       <x:c r="A18" s="16" t="str">
@@ -2317,30 +2345,30 @@
       <x:c r="B18" s="16" t="str">
         <x:v>安装人员</x:v>
       </x:c>
-      <x:c r="C18" s="45" t="str">
+      <x:c r="C18" s="51" t="str">
         <x:v>待安排</x:v>
       </x:c>
-      <x:c r="D18" s="45"/>
+      <x:c r="D18" s="51"/>
       <x:c r="E18" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
       <x:c r="F18" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
-      <x:c r="G18" s="45" t="str">
+      <x:c r="G18" s="51" t="str">
         <x:v>待确定</x:v>
       </x:c>
-      <x:c r="H18" s="45"/>
+      <x:c r="H18" s="51"/>
       <x:c r="I18" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
       <x:c r="J18" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
-      <x:c r="K18" s="45" t="str">
+      <x:c r="K18" s="51" t="str">
         <x:v>待确认</x:v>
       </x:c>
-      <x:c r="L18" s="45"/>
+      <x:c r="L18" s="51"/>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="15" t="str">
@@ -2387,30 +2415,30 @@
       <x:c r="B20" s="16" t="str">
         <x:v>产品名称 / 编号</x:v>
       </x:c>
-      <x:c r="C20" s="45" t="str">
+      <x:c r="C20" s="51" t="str">
         <x:v>控制器 C05</x:v>
       </x:c>
-      <x:c r="D20" s="45"/>
+      <x:c r="D20" s="51"/>
       <x:c r="E20" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
       <x:c r="F20" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
-      <x:c r="G20" s="46" t="d">
+      <x:c r="G20" s="52" t="d">
         <x:v>2026-05-20T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="H20" s="46"/>
+      <x:c r="H20" s="52"/>
       <x:c r="I20" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
       <x:c r="J20" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
-      <x:c r="K20" s="45" t="str">
+      <x:c r="K20" s="51" t="str">
         <x:v>设备故障</x:v>
       </x:c>
-      <x:c r="L20" s="45"/>
+      <x:c r="L20" s="51"/>
     </x:row>
     <x:row r="21" ht="31" customHeight="1">
       <x:c r="A21" s="16" t="str">
@@ -2419,30 +2447,30 @@
       <x:c r="B21" s="16" t="str">
         <x:v>问题等级</x:v>
       </x:c>
-      <x:c r="C21" s="45" t="str">
+      <x:c r="C21" s="51" t="str">
         <x:v>待评估</x:v>
       </x:c>
-      <x:c r="D21" s="45"/>
+      <x:c r="D21" s="51"/>
       <x:c r="E21" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
       <x:c r="F21" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
-      <x:c r="G21" s="47" t="str">
+      <x:c r="G21" s="53" t="str">
         <x:v>李售后</x:v>
       </x:c>
-      <x:c r="H21" s="47"/>
+      <x:c r="H21" s="53"/>
       <x:c r="I21" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
       <x:c r="J21" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
-      <x:c r="K21" s="46" t="d">
+      <x:c r="K21" s="52" t="d">
         <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="L21" s="46"/>
+      <x:c r="L21" s="52"/>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="16" t="str">
@@ -2451,18 +2479,18 @@
       <x:c r="B22" s="16" t="str">
         <x:v>问题描述 *</x:v>
       </x:c>
-      <x:c r="C22" s="47" t="str">
+      <x:c r="C22" s="53" t="str">
         <x:v>同一项目另一台设备无法启动，指示灯常亮。</x:v>
       </x:c>
-      <x:c r="D22" s="47"/>
-      <x:c r="E22" s="47"/>
-      <x:c r="F22" s="47"/>
-      <x:c r="G22" s="47"/>
-      <x:c r="H22" s="47"/>
-      <x:c r="I22" s="47"/>
-      <x:c r="J22" s="47"/>
-      <x:c r="K22" s="47"/>
-      <x:c r="L22" s="47"/>
+      <x:c r="D22" s="53"/>
+      <x:c r="E22" s="53"/>
+      <x:c r="F22" s="53"/>
+      <x:c r="G22" s="53"/>
+      <x:c r="H22" s="53"/>
+      <x:c r="I22" s="53"/>
+      <x:c r="J22" s="53"/>
+      <x:c r="K22" s="53"/>
+      <x:c r="L22" s="53"/>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" s="16" t="str">
@@ -2471,20 +2499,20 @@
       <x:c r="B23" s="16" t="str">
         <x:v>客户反馈 / 当前处理记录</x:v>
       </x:c>
-      <x:c r="C23" s="45" t="str">
+      <x:c r="C23" s="51" t="str">
         <x:v>已收到客户反馈，与电机问题分开跟踪。</x:v>
       </x:c>
-      <x:c r="D23" s="45"/>
-      <x:c r="E23" s="45"/>
-      <x:c r="F23" s="45"/>
-      <x:c r="G23" s="45"/>
-      <x:c r="H23" s="45"/>
+      <x:c r="D23" s="51"/>
+      <x:c r="E23" s="51"/>
+      <x:c r="F23" s="51"/>
+      <x:c r="G23" s="51"/>
+      <x:c r="H23" s="51"/>
       <x:c r="I23" s="22" t="str">
         <x:v>售后原因</x:v>
       </x:c>
       <x:c r="J23" s="22"/>
-      <x:c r="K23" s="45"/>
-      <x:c r="L23" s="45"/>
+      <x:c r="K23" s="51"/>
+      <x:c r="L23" s="51"/>
     </x:row>
     <x:row r="24" ht="135" customHeight="1">
       <x:c r="A24" s="16" t="str">
@@ -2493,22 +2521,22 @@
       <x:c r="B24" s="16" t="str">
         <x:v>附件提供方式</x:v>
       </x:c>
-      <x:c r="C24" s="45" t="str">
+      <x:c r="C24" s="51" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
-      <x:c r="D24" s="45"/>
+      <x:c r="D24" s="51"/>
       <x:c r="E24" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
       <x:c r="F24" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
-      <x:c r="G24" s="45"/>
-      <x:c r="H24" s="45"/>
-      <x:c r="I24" s="45"/>
-      <x:c r="J24" s="45"/>
-      <x:c r="K24" s="45"/>
-      <x:c r="L24" s="45"/>
+      <x:c r="G24" s="51"/>
+      <x:c r="H24" s="51"/>
+      <x:c r="I24" s="51"/>
+      <x:c r="J24" s="51"/>
+      <x:c r="K24" s="51"/>
+      <x:c r="L24" s="51"/>
     </x:row>
     <x:row r="25" ht="31" customHeight="1">
       <x:c r="A25" s="16" t="str">
@@ -2517,28 +2545,28 @@
       <x:c r="B25" s="16" t="str">
         <x:v>当前阶段</x:v>
       </x:c>
-      <x:c r="C25" s="45" t="str">
+      <x:c r="C25" s="51" t="str">
         <x:v>审核</x:v>
       </x:c>
-      <x:c r="D25" s="45"/>
+      <x:c r="D25" s="51"/>
       <x:c r="E25" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
       <x:c r="F25" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
-      <x:c r="G25" s="46"/>
-      <x:c r="H25" s="46"/>
+      <x:c r="G25" s="52"/>
+      <x:c r="H25" s="52"/>
       <x:c r="I25" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
       <x:c r="J25" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
-      <x:c r="K25" s="45" t="str">
+      <x:c r="K25" s="51" t="str">
         <x:v>确认设备接线及状态</x:v>
       </x:c>
-      <x:c r="L25" s="45"/>
+      <x:c r="L25" s="51"/>
     </x:row>
     <x:row r="26" ht="31" customHeight="1">
       <x:c r="A26" s="16" t="str">
@@ -2547,30 +2575,30 @@
       <x:c r="B26" s="16" t="str">
         <x:v>商务</x:v>
       </x:c>
-      <x:c r="C26" s="45" t="str">
+      <x:c r="C26" s="51" t="str">
         <x:v>林商务</x:v>
       </x:c>
-      <x:c r="D26" s="45"/>
+      <x:c r="D26" s="51"/>
       <x:c r="E26" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
       <x:c r="F26" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
-      <x:c r="G26" s="45" t="str">
+      <x:c r="G26" s="51" t="str">
         <x:v>陈设计</x:v>
       </x:c>
-      <x:c r="H26" s="45"/>
+      <x:c r="H26" s="51"/>
       <x:c r="I26" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
       <x:c r="J26" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
-      <x:c r="K26" s="45" t="str">
+      <x:c r="K26" s="51" t="str">
         <x:v>周工程</x:v>
       </x:c>
-      <x:c r="L26" s="45"/>
+      <x:c r="L26" s="51"/>
     </x:row>
     <x:row r="27" ht="31" customHeight="1">
       <x:c r="A27" s="16" t="str">
@@ -2579,28 +2607,28 @@
       <x:c r="B27" s="16" t="str">
         <x:v>安装人员</x:v>
       </x:c>
-      <x:c r="C27" s="45"/>
-      <x:c r="D27" s="45"/>
+      <x:c r="C27" s="51"/>
+      <x:c r="D27" s="51"/>
       <x:c r="E27" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
       <x:c r="F27" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
-      <x:c r="G27" s="45" t="str">
+      <x:c r="G27" s="51" t="str">
         <x:v>待确定</x:v>
       </x:c>
-      <x:c r="H27" s="45"/>
+      <x:c r="H27" s="51"/>
       <x:c r="I27" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
       <x:c r="J27" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
-      <x:c r="K27" s="45" t="str">
+      <x:c r="K27" s="51" t="str">
         <x:v>待确认</x:v>
       </x:c>
-      <x:c r="L27" s="45"/>
+      <x:c r="L27" s="51"/>
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="15" t="str">
@@ -2647,28 +2675,28 @@
       <x:c r="B29" s="16" t="str">
         <x:v>产品名称 / 编号</x:v>
       </x:c>
-      <x:c r="C29" s="45" t="str">
+      <x:c r="C29" s="51" t="str">
         <x:v>护板 P06</x:v>
       </x:c>
-      <x:c r="D29" s="45"/>
+      <x:c r="D29" s="51"/>
       <x:c r="E29" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
       <x:c r="F29" s="16" t="str">
         <x:v>设备交付日期</x:v>
       </x:c>
-      <x:c r="G29" s="46"/>
-      <x:c r="H29" s="46"/>
+      <x:c r="G29" s="52"/>
+      <x:c r="H29" s="52"/>
       <x:c r="I29" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
       <x:c r="J29" s="16" t="str">
         <x:v>问题分类</x:v>
       </x:c>
-      <x:c r="K29" s="45" t="str">
+      <x:c r="K29" s="51" t="str">
         <x:v>外观破损</x:v>
       </x:c>
-      <x:c r="L29" s="45"/>
+      <x:c r="L29" s="51"/>
     </x:row>
     <x:row r="30" ht="31" customHeight="1">
       <x:c r="A30" s="16" t="str">
@@ -2677,28 +2705,28 @@
       <x:c r="B30" s="16" t="str">
         <x:v>问题等级</x:v>
       </x:c>
-      <x:c r="C30" s="45" t="str">
+      <x:c r="C30" s="51" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D30" s="45"/>
+      <x:c r="D30" s="51"/>
       <x:c r="E30" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
       <x:c r="F30" s="16" t="str">
         <x:v>售后负责人 *</x:v>
       </x:c>
-      <x:c r="G30" s="47" t="str">
+      <x:c r="G30" s="53" t="str">
         <x:v>张售后</x:v>
       </x:c>
-      <x:c r="H30" s="47"/>
+      <x:c r="H30" s="53"/>
       <x:c r="I30" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
       <x:c r="J30" s="16" t="str">
         <x:v>计划完成时间</x:v>
       </x:c>
-      <x:c r="K30" s="46"/>
-      <x:c r="L30" s="46"/>
+      <x:c r="K30" s="52"/>
+      <x:c r="L30" s="52"/>
     </x:row>
     <x:row r="31" ht="48" customHeight="1">
       <x:c r="A31" s="16" t="str">
@@ -2707,18 +2735,18 @@
       <x:c r="B31" s="16" t="str">
         <x:v>问题描述 *</x:v>
       </x:c>
-      <x:c r="C31" s="47" t="str">
+      <x:c r="C31" s="53" t="str">
         <x:v>护板表面破损，设备交付日期待核实。</x:v>
       </x:c>
-      <x:c r="D31" s="47"/>
-      <x:c r="E31" s="47"/>
-      <x:c r="F31" s="47"/>
-      <x:c r="G31" s="47"/>
-      <x:c r="H31" s="47"/>
-      <x:c r="I31" s="47"/>
-      <x:c r="J31" s="47"/>
-      <x:c r="K31" s="47"/>
-      <x:c r="L31" s="47"/>
+      <x:c r="D31" s="53"/>
+      <x:c r="E31" s="53"/>
+      <x:c r="F31" s="53"/>
+      <x:c r="G31" s="53"/>
+      <x:c r="H31" s="53"/>
+      <x:c r="I31" s="53"/>
+      <x:c r="J31" s="53"/>
+      <x:c r="K31" s="53"/>
+      <x:c r="L31" s="53"/>
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
       <x:c r="A32" s="16" t="str">
@@ -2727,20 +2755,20 @@
       <x:c r="B32" s="16" t="str">
         <x:v>客户反馈 / 当前处理记录</x:v>
       </x:c>
-      <x:c r="C32" s="45" t="str">
+      <x:c r="C32" s="51" t="str">
         <x:v>请商务补充本台设备的实际交付记录。</x:v>
       </x:c>
-      <x:c r="D32" s="45"/>
-      <x:c r="E32" s="45"/>
-      <x:c r="F32" s="45"/>
-      <x:c r="G32" s="45"/>
-      <x:c r="H32" s="45"/>
+      <x:c r="D32" s="51"/>
+      <x:c r="E32" s="51"/>
+      <x:c r="F32" s="51"/>
+      <x:c r="G32" s="51"/>
+      <x:c r="H32" s="51"/>
       <x:c r="I32" s="22" t="str">
         <x:v>售后原因</x:v>
       </x:c>
       <x:c r="J32" s="22"/>
-      <x:c r="K32" s="45"/>
-      <x:c r="L32" s="45"/>
+      <x:c r="K32" s="51"/>
+      <x:c r="L32" s="51"/>
     </x:row>
     <x:row r="33" ht="135" customHeight="1">
       <x:c r="A33" s="16" t="str">
@@ -2749,20 +2777,20 @@
       <x:c r="B33" s="16" t="str">
         <x:v>附件提供方式</x:v>
       </x:c>
-      <x:c r="C33" s="45"/>
-      <x:c r="D33" s="45"/>
+      <x:c r="C33" s="51"/>
+      <x:c r="D33" s="51"/>
       <x:c r="E33" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
       <x:c r="F33" s="16" t="str">
         <x:v>照片 / 视频链接</x:v>
       </x:c>
-      <x:c r="G33" s="45"/>
-      <x:c r="H33" s="45"/>
-      <x:c r="I33" s="45"/>
-      <x:c r="J33" s="45"/>
-      <x:c r="K33" s="45"/>
-      <x:c r="L33" s="45"/>
+      <x:c r="G33" s="51"/>
+      <x:c r="H33" s="51"/>
+      <x:c r="I33" s="51"/>
+      <x:c r="J33" s="51"/>
+      <x:c r="K33" s="51"/>
+      <x:c r="L33" s="51"/>
     </x:row>
     <x:row r="34" ht="31" customHeight="1">
       <x:c r="A34" s="16" t="str">
@@ -2771,26 +2799,26 @@
       <x:c r="B34" s="16" t="str">
         <x:v>当前阶段</x:v>
       </x:c>
-      <x:c r="C34" s="45" t="str">
+      <x:c r="C34" s="51" t="str">
         <x:v>审核</x:v>
       </x:c>
-      <x:c r="D34" s="45"/>
+      <x:c r="D34" s="51"/>
       <x:c r="E34" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
       <x:c r="F34" s="16" t="str">
         <x:v>实际完成时间</x:v>
       </x:c>
-      <x:c r="G34" s="46"/>
-      <x:c r="H34" s="46"/>
+      <x:c r="G34" s="52"/>
+      <x:c r="H34" s="52"/>
       <x:c r="I34" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
       <x:c r="J34" s="16" t="str">
         <x:v>下一步</x:v>
       </x:c>
-      <x:c r="K34" s="45"/>
-      <x:c r="L34" s="45"/>
+      <x:c r="K34" s="51"/>
+      <x:c r="L34" s="51"/>
     </x:row>
     <x:row r="35" ht="31" customHeight="1">
       <x:c r="A35" s="16" t="str">
@@ -2799,24 +2827,24 @@
       <x:c r="B35" s="16" t="str">
         <x:v>商务</x:v>
       </x:c>
-      <x:c r="C35" s="45"/>
-      <x:c r="D35" s="45"/>
+      <x:c r="C35" s="51"/>
+      <x:c r="D35" s="51"/>
       <x:c r="E35" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
       <x:c r="F35" s="16" t="str">
         <x:v>设计师</x:v>
       </x:c>
-      <x:c r="G35" s="45"/>
-      <x:c r="H35" s="45"/>
+      <x:c r="G35" s="51"/>
+      <x:c r="H35" s="51"/>
       <x:c r="I35" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
       <x:c r="J35" s="16" t="str">
         <x:v>工程师</x:v>
       </x:c>
-      <x:c r="K35" s="45"/>
-      <x:c r="L35" s="45"/>
+      <x:c r="K35" s="51"/>
+      <x:c r="L35" s="51"/>
     </x:row>
     <x:row r="36" ht="31" customHeight="1">
       <x:c r="A36" s="16" t="str">
@@ -2825,28 +2853,28 @@
       <x:c r="B36" s="16" t="str">
         <x:v>安装人员</x:v>
       </x:c>
-      <x:c r="C36" s="45"/>
-      <x:c r="D36" s="45"/>
+      <x:c r="C36" s="51"/>
+      <x:c r="D36" s="51"/>
       <x:c r="E36" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
       <x:c r="F36" s="16" t="str">
         <x:v>执行方式</x:v>
       </x:c>
-      <x:c r="G36" s="45" t="str">
+      <x:c r="G36" s="51" t="str">
         <x:v>待确定</x:v>
       </x:c>
-      <x:c r="H36" s="45"/>
+      <x:c r="H36" s="51"/>
       <x:c r="I36" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
       <x:c r="J36" s="16" t="str">
         <x:v>费用承担</x:v>
       </x:c>
-      <x:c r="K36" s="45" t="str">
+      <x:c r="K36" s="51" t="str">
         <x:v>待确认</x:v>
       </x:c>
-      <x:c r="L36" s="45"/>
+      <x:c r="L36" s="51"/>
     </x:row>
     <x:row r="37" ht="27" customHeight="1">
       <x:c r="A37" s="6" t="str">
@@ -3092,7 +3120,7 @@
       <x:formula1>"待评估,S,A,B,C"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K14:L14">
-      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏"</x:formula1>
+      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏,正常损耗"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C15:D15">
       <x:formula1>"上传照片 / 视频,照片 / 视频链接"</x:formula1>
@@ -3113,7 +3141,7 @@
       <x:formula1>"待评估,S,A,B,C"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K23:L23">
-      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏"</x:formula1>
+      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏,正常损耗"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C24:D24">
       <x:formula1>"上传照片 / 视频,照片 / 视频链接"</x:formula1>
@@ -3134,7 +3162,7 @@
       <x:formula1>"待评估,S,A,B,C"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K32:L32">
-      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏"</x:formula1>
+      <x:formula1>"待确认,安装缺陷,设计缺陷,工程下单缺陷,生产缺陷,人为损坏,正常损耗"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C33:D33">
       <x:formula1>"上传照片 / 视频,照片 / 视频链接"</x:formula1>

</xml_diff>